<commit_message>
[feat][Inventory] Inventory 및 아이템 습득 사용 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Item.xlsx
+++ b/JsonConverter/ExcelFiles/Item.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t xml:space="preserve">캐릭터 고유 ID</t>
   </si>
@@ -31,6 +31,9 @@
     <t xml:space="preserve">string</t>
   </si>
   <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
     <t xml:space="preserve">Id</t>
   </si>
   <si>
@@ -43,13 +46,19 @@
     <t xml:space="preserve">IconPath</t>
   </si>
   <si>
+    <t xml:space="preserve">UseType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UseValue</t>
+  </si>
+  <si>
     <t xml:space="preserve">Item_0001</t>
   </si>
   <si>
-    <t xml:space="preserve">아이템 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">아이템 1의 설명</t>
+    <t xml:space="preserve">+30HP 포션</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+30HP 포션 이다</t>
   </si>
   <si>
     <r>
@@ -74,32 +83,16 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Heal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Item_0002</t>
   </si>
   <si>
-    <t xml:space="preserve">아이템 2</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">아이템 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">의 설명</t>
-    </r>
+    <t xml:space="preserve">+50HP 포션</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+50HP 포션 이다</t>
   </si>
   <si>
     <t xml:space="preserve">Icon/Icon_Item_Item_0002</t>
@@ -108,29 +101,10 @@
     <t xml:space="preserve">Item_0003</t>
   </si>
   <si>
-    <t xml:space="preserve">아이템 3</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">아이템 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">의 설명</t>
-    </r>
+    <t xml:space="preserve">+100HP 포션</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+100HP 포션 이다</t>
   </si>
   <si>
     <t xml:space="preserve">Icon/Icon_Item_Item_0003</t>
@@ -139,32 +113,16 @@
     <t xml:space="preserve">Item_0004</t>
   </si>
   <si>
-    <t xml:space="preserve">아이템 4</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">아이템 4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="&quot;맑은 고딕&quot;"/>
-        <family val="0"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">의 설명</t>
-    </r>
+    <t xml:space="preserve">-50HP 포션</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-50HP 포션 이다</t>
   </si>
   <si>
     <t xml:space="preserve">Icon/Icon_Item_Item_0004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TakeDamage</t>
   </si>
   <si>
     <t xml:space="preserve">Item_0005</t>
@@ -198,6 +156,9 @@
     <t xml:space="preserve">Icon/Icon_Item_Item_0005</t>
   </si>
   <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
     <t xml:space="preserve">Item_0006</t>
   </si>
   <si>
@@ -267,7 +228,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -301,6 +262,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="129"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF008000"/>
       <name val="&quot;맑은 고딕&quot;"/>
@@ -320,6 +288,12 @@
       <name val="&quot;맑은 고딕&quot;"/>
       <family val="0"/>
       <charset val="129"/>
+    </font>
+    <font>
+      <sz val="9.5"/>
+      <color rgb="FF000000"/>
+      <name val="DotumChe"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="4">
@@ -383,7 +357,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -396,11 +370,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -412,7 +394,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -674,7 +668,7 @@
   <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.05"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="5" style="1" width="10.58"/>
@@ -701,312 +695,353 @@
       <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" s="5" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="E2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+    </row>
+    <row r="3" s="7" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="6"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="0"/>
+      <c r="D3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="F5" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+        <v>19</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+        <v>23</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+        <v>30</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+      <c r="F10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
+      <c r="A35" s="9"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>